<commit_message>
feat: Add notification banner on accepted PRN/PERN
- adds notification banner shared component macro
- includes "Success" notification on prn/pern acceptance
- shared buttons for pre and post acceptance state
- download/print PDF added
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
+++ b/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="167">
   <si>
     <t>Translator notes</t>
   </si>
@@ -376,6 +376,60 @@
     <t>Mae'r PRN yma yn ymwneud â gwastraff a gafodd ei allforio i'w ailbrosesu ym mis Rhagfyr {{year}}.</t>
   </si>
   <si>
+    <t>prns.prn.acceptOrRejectMoreButton</t>
+  </si>
+  <si>
+    <t>Accept or reject more PRNs and PERNs for {{year}}</t>
+  </si>
+  <si>
+    <t>prns.prn.acceptOrRejectMoreButtonNoYear</t>
+  </si>
+  <si>
+    <t>Accept or reject more PRNs and PERNs</t>
+  </si>
+  <si>
+    <t>prns.prn.obligationProgressButton</t>
+  </si>
+  <si>
+    <t>View your {{year}} recycling obligations progress</t>
+  </si>
+  <si>
+    <t>prns.prn.obligationProgressButtonNoYear</t>
+  </si>
+  <si>
+    <t>View your recycling obligations progress</t>
+  </si>
+  <si>
+    <t>prns.prn.downloadThisAcceptedPrn</t>
+  </si>
+  <si>
+    <t>prns.prn.downloadThisAcceptedPern</t>
+  </si>
+  <si>
+    <t>prns.prn.success.title</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>prns.prn.success.heading</t>
+  </si>
+  <si>
+    <t>You accepted this {{type}} towards your {{year}} recycling obligations</t>
+  </si>
+  <si>
+    <t>prns.prn.success.description-one-tonne</t>
+  </si>
+  <si>
+    <t>You have accepted {{tonnage}} tonne towards your {{year}} recycling obligation for {{material}} material.</t>
+  </si>
+  <si>
+    <t>prns.prn.success.description</t>
+  </si>
+  <si>
+    <t>You have accepted {{tonnage}} tonnes towards your {{year}} recycling obligation for {{material}} material.</t>
+  </si>
+  <si>
     <t>prns.prn.agency.ea</t>
   </si>
   <si>
@@ -452,6 +506,12 @@
   </si>
   <si>
     <t>has accepted the {{prnOrPern}}.</t>
+  </si>
+  <si>
+    <t>prns.prn.success.headingNoYear</t>
+  </si>
+  <si>
+    <t>You accepted this {{type}} towards your recycling obligations</t>
   </si>
 </sst>
 </file>
@@ -850,7 +910,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -1792,7 +1852,7 @@
         <v>11</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>130</v>
+        <v>90</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>13</v>
@@ -1803,7 +1863,7 @@
     </row>
     <row r="51" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>10</v>
@@ -1812,7 +1872,7 @@
         <v>11</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>132</v>
+        <v>93</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>13</v>
@@ -1823,7 +1883,7 @@
     </row>
     <row r="52" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>10</v>
@@ -1832,7 +1892,7 @@
         <v>11</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>13</v>
@@ -1843,7 +1903,7 @@
     </row>
     <row r="53" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>10</v>
@@ -1852,7 +1912,7 @@
         <v>11</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>13</v>
@@ -1863,36 +1923,36 @@
     </row>
     <row r="54" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D54" s="1" t="s">
+      <c r="B55" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D55" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="55" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>13</v>
@@ -1903,7 +1963,7 @@
     </row>
     <row r="56" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>10</v>
@@ -1912,7 +1972,7 @@
         <v>11</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>13</v>
@@ -1923,7 +1983,7 @@
     </row>
     <row r="57" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>10</v>
@@ -1932,7 +1992,7 @@
         <v>11</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>13</v>
@@ -1943,26 +2003,246 @@
     </row>
     <row r="58" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="59" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B58" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D58" s="1" t="s">
+      <c r="B59" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="E58" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F58" s="1" t="s">
+      <c r="E59" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="61" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="62" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="63" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="64" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="65" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="67" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="68" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="69" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F69" s="1" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:F58"/>
+  <autoFilter ref="A5:F69"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
feat: MO-479 show December waste flash on PRN pages
Show a blue "Can be accepted towards {yearOne} or {yearTwo}" flash on awaiting-acceptance December waste PRNs that offer a choice of two available acceptance years, during the UK December/January window. Shown on the
producer and CSO PRN detail pages and the PRNs list; the PRN routes are already behind the epic flag FEATURE_SHOW_PRNS.

- add getUkYearMonth for UK (Europe/London) year/month

- add the flash window rules and buildDecemberWasteFlash

- add the prn-flash-label component

- use {{yearOne}}/{{yearTwo}} in the two-year copy and regenerate the Welsh exports
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
+++ b/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="166">
   <si>
     <t>Translator notes</t>
   </si>
@@ -322,16 +322,10 @@
     <t>Lawrlwytho'r PERN yma sy'n aros i gael ei dderbyn fel PDF</t>
   </si>
   <si>
-    <t>prns.prn.acceptanceYear</t>
-  </si>
-  <si>
-    <t>Can be accepted towards {{year}}</t>
-  </si>
-  <si>
     <t>prns.prn.acceptanceYears</t>
   </si>
   <si>
-    <t>Can be accepted towards {{year}} or {{year}}</t>
+    <t>Can be accepted towards {{yearOne}} or {{yearTwo}}</t>
   </si>
   <si>
     <t>prns.prn.acceptedTowardsRecyclingObligations</t>
@@ -913,7 +907,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -1635,7 +1629,7 @@
         <v>11</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>13</v>
@@ -1646,19 +1640,19 @@
     </row>
     <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="E40" s="1" t="s">
-        <v>13</v>
+        <v>108</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>13</v>
@@ -1666,7 +1660,7 @@
     </row>
     <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>10</v>
@@ -1675,10 +1669,10 @@
         <v>11</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>13</v>
@@ -1686,7 +1680,7 @@
     </row>
     <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>10</v>
@@ -1695,10 +1689,10 @@
         <v>11</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>13</v>
@@ -1706,7 +1700,7 @@
     </row>
     <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>10</v>
@@ -1715,10 +1709,10 @@
         <v>11</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>13</v>
@@ -1726,19 +1720,19 @@
     </row>
     <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>80</v>
-      </c>
       <c r="E44" s="1" t="s">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>13</v>
@@ -1746,7 +1740,7 @@
     </row>
     <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>10</v>
@@ -1755,10 +1749,10 @@
         <v>11</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>13</v>
@@ -1766,7 +1760,7 @@
     </row>
     <row r="46" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>10</v>
@@ -1775,10 +1769,10 @@
         <v>11</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>121</v>
+        <v>13</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>13</v>
@@ -1855,7 +1849,7 @@
         <v>11</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>129</v>
+        <v>92</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>13</v>
@@ -1866,7 +1860,7 @@
     </row>
     <row r="51" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>10</v>
@@ -1875,7 +1869,7 @@
         <v>11</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>13</v>
@@ -1886,16 +1880,16 @@
     </row>
     <row r="52" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D52" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>13</v>
@@ -1924,7 +1918,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>134</v>
       </c>
@@ -1964,7 +1958,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>138</v>
       </c>
@@ -2124,7 +2118,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>154</v>
       </c>
@@ -2144,7 +2138,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="65" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>156</v>
       </c>
@@ -2244,28 +2238,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="70" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:F70"/>
+  <autoFilter ref="A5:F69"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
MO-442: Added support for generating PDF downloads of PRNs
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
+++ b/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="178">
   <si>
     <t>Translator notes</t>
   </si>
@@ -427,6 +427,15 @@
     <t>You have accepted {{tonnage}} tonnes towards your {{year}} recycling obligation for {{material}} material.</t>
   </si>
   <si>
+    <t>prns.prn.rejected.heading</t>
+  </si>
+  <si>
+    <t>{{type}} rejected.</t>
+  </si>
+  <si>
+    <t>{{type}} rwrthod</t>
+  </si>
+  <si>
     <t>prns.prn.agency.ea</t>
   </si>
   <si>
@@ -503,6 +512,33 @@
   </si>
   <si>
     <t>has accepted the {{prnOrPern}}.</t>
+  </si>
+  <si>
+    <t>prns.prn.pdf.awaitingCancellation</t>
+  </si>
+  <si>
+    <t>Awaiting cancellation</t>
+  </si>
+  <si>
+    <t>Yn aros i gael ei ganslo</t>
+  </si>
+  <si>
+    <t>prns.prn.pdf.rejectedMeaning</t>
+  </si>
+  <si>
+    <t>The producer or compliance scheme rejected this {{prnOrPern}}. The reprocessor or exporter has not yet cancelled it.</t>
+  </si>
+  <si>
+    <t>Cafodd y PRN yma ei wrthod gan y cynhyrchydd neu'r cynllun cydymffurfio. Dyw'r ailbrosesydd neu'r allforiwr ddim wedi'i ganslo eto</t>
+  </si>
+  <si>
+    <t>prns.prn.pdf.tonnageInWords</t>
+  </si>
+  <si>
+    <t>Tonnage in words</t>
+  </si>
+  <si>
+    <t>Tunelli mewn geiriau</t>
   </si>
   <si>
     <t>prns.prn.success.headingNoYear</t>
@@ -907,7 +943,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -1972,7 +2008,7 @@
         <v>139</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>13</v>
+        <v>140</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>13</v>
@@ -1980,7 +2016,7 @@
     </row>
     <row r="57" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>10</v>
@@ -1989,7 +2025,7 @@
         <v>11</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>13</v>
@@ -2000,7 +2036,7 @@
     </row>
     <row r="58" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>10</v>
@@ -2009,7 +2045,7 @@
         <v>11</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>13</v>
@@ -2020,7 +2056,7 @@
     </row>
     <row r="59" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>10</v>
@@ -2029,7 +2065,7 @@
         <v>11</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>13</v>
@@ -2040,7 +2076,7 @@
     </row>
     <row r="60" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>10</v>
@@ -2049,7 +2085,7 @@
         <v>11</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>13</v>
@@ -2060,7 +2096,7 @@
     </row>
     <row r="61" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>10</v>
@@ -2069,7 +2105,7 @@
         <v>11</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>13</v>
@@ -2080,7 +2116,7 @@
     </row>
     <row r="62" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>10</v>
@@ -2089,7 +2125,7 @@
         <v>11</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>13</v>
@@ -2100,7 +2136,7 @@
     </row>
     <row r="63" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>10</v>
@@ -2109,7 +2145,7 @@
         <v>11</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>13</v>
@@ -2118,9 +2154,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>10</v>
@@ -2129,7 +2165,7 @@
         <v>11</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>13</v>
@@ -2138,9 +2174,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="65" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>10</v>
@@ -2149,7 +2185,7 @@
         <v>11</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>13</v>
@@ -2160,7 +2196,7 @@
     </row>
     <row r="66" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>10</v>
@@ -2169,7 +2205,7 @@
         <v>11</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>13</v>
@@ -2180,7 +2216,7 @@
     </row>
     <row r="67" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>10</v>
@@ -2189,7 +2225,7 @@
         <v>11</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>13</v>
@@ -2200,7 +2236,7 @@
     </row>
     <row r="68" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>10</v>
@@ -2209,7 +2245,7 @@
         <v>11</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>13</v>
@@ -2220,7 +2256,7 @@
     </row>
     <row r="69" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>10</v>
@@ -2229,7 +2265,7 @@
         <v>11</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>13</v>
@@ -2238,8 +2274,88 @@
         <v>13</v>
       </c>
     </row>
+    <row r="70" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="71" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="73" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:F69"/>
+  <autoFilter ref="A5:F73"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>

<commit_message>
MO-469: Enhance PRN rejection confirmation functionality
- Updated the confirmation page to include a form for submitting rejection.
- Modified the PRN status handling to allow rejection and redirect to the appropriate confirmation page.
- Improved UI elements to reflect the rejection status and updated related translations.
- Added tests to ensure the rejection process works as intended and handles edge cases correctly.
- Refactored existing routes to streamline the rejection confirmation logic.
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
+++ b/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="177">
   <si>
     <t>Translator notes</t>
   </si>
@@ -181,7 +181,7 @@
     <t>prns.prn.relatesToWasteReceivedInDecember</t>
   </si>
   <si>
-    <t>December Waste?</t>
+    <t>December waste?</t>
   </si>
   <si>
     <t>Gwastraff Rhagfyr?</t>
@@ -190,7 +190,7 @@
     <t>prns.prn.isDecemberWaste</t>
   </si>
   <si>
-    <t>yes</t>
+    <t>Yes</t>
   </si>
   <si>
     <t>Ydw</t>
@@ -199,7 +199,7 @@
     <t>prns.prn.isNotDecemberWaste</t>
   </si>
   <si>
-    <t>no</t>
+    <t>No</t>
   </si>
   <si>
     <t>Nac ydw</t>
@@ -289,120 +289,120 @@
     <t>prns.prn.downloadThisPrn</t>
   </si>
   <si>
+    <t>Download this PRN as a PDF or HTML</t>
+  </si>
+  <si>
+    <t>prns.prn.downloadThisPern</t>
+  </si>
+  <si>
+    <t>Download this PERN as a PDF or HTML</t>
+  </si>
+  <si>
+    <t>prns.prn.downloadThisPrnAwaitingAcceptance</t>
+  </si>
+  <si>
+    <t>Download this awaiting acceptance PRN as a PDF</t>
+  </si>
+  <si>
+    <t>Lawrlwytho'r PRN yma sy'n aros i gael ei dderbyn fel PDF</t>
+  </si>
+  <si>
+    <t>prns.prn.downloadThisPernAwaitingAcceptance</t>
+  </si>
+  <si>
+    <t>Download this awaiting acceptance PERN as a PDF</t>
+  </si>
+  <si>
+    <t>Lawrlwytho'r PERN yma sy'n aros i gael ei dderbyn fel PDF</t>
+  </si>
+  <si>
+    <t>prns.prn.acceptanceYears</t>
+  </si>
+  <si>
+    <t>Can be accepted towards {{yearOne}} or {{yearTwo}}</t>
+  </si>
+  <si>
+    <t>prns.prn.acceptedTowardsRecyclingObligations</t>
+  </si>
+  <si>
+    <t>prns.prn.note</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Nodi</t>
+  </si>
+  <si>
+    <t>prns.prn.packagingExportRecyclingNote</t>
+  </si>
+  <si>
+    <t>Packaging Waste Export Recycling Note</t>
+  </si>
+  <si>
+    <t>Nodyn Ailgylchu Allforio Gwastraff Pecynwaith</t>
+  </si>
+  <si>
+    <t>prns.prn.pageTitlePern</t>
+  </si>
+  <si>
+    <t>prns.prn.pageTitlePrn</t>
+  </si>
+  <si>
+    <t>prns.prn.thisPernRelatesToWasteExportedForReprocessingInDecember</t>
+  </si>
+  <si>
+    <t>This PERN relates to waste exported for reprocessing in December {{year}}.</t>
+  </si>
+  <si>
+    <t>Mae'r PERN yma yn ymwneud â gwastraff a gafodd ei allforio i'w ailbrosesu ym mis Rhagfyr {{year}}.</t>
+  </si>
+  <si>
+    <t>prns.prn.thisPrnRelatesToWasteReceivedForReprocessingInDecember</t>
+  </si>
+  <si>
+    <t>This PRN relates to waste received for reprocessing in December {{year}}.</t>
+  </si>
+  <si>
+    <t>Mae'r PRN yma yn ymwneud â gwastraff a gafodd ei allforio i'w ailbrosesu ym mis Rhagfyr {{year}}.</t>
+  </si>
+  <si>
+    <t>prns.prn.acceptOrRejectMoreButton</t>
+  </si>
+  <si>
+    <t>Accept or reject more PRNs and PERNs for {{year}}</t>
+  </si>
+  <si>
+    <t>prns.prn.acceptOrRejectMoreButtonNoYear</t>
+  </si>
+  <si>
+    <t>Accept or reject more PRNs and PERNs</t>
+  </si>
+  <si>
+    <t>prns.prn.obligationProgressButton</t>
+  </si>
+  <si>
+    <t>View your {{year}} recycling obligations progress</t>
+  </si>
+  <si>
+    <t>prns.prn.obligationProgressButtonNoYear</t>
+  </si>
+  <si>
+    <t>View your recycling obligations progress</t>
+  </si>
+  <si>
+    <t>prns.prn.downloadThisAcceptedPrn</t>
+  </si>
+  <si>
     <t>Download this PRN as a PDF</t>
   </si>
   <si>
-    <t>Lawrlwytho'r PRN yma fel PDF</t>
-  </si>
-  <si>
-    <t>prns.prn.downloadThisPern</t>
+    <t>prns.prn.downloadThisAcceptedPern</t>
   </si>
   <si>
     <t>Download this PERN as a PDF</t>
   </si>
   <si>
-    <t>Lawrlwytho'r PERN yma fel PDF</t>
-  </si>
-  <si>
-    <t>prns.prn.downloadThisPrnAwaitingAcceptance</t>
-  </si>
-  <si>
-    <t>Download this awaiting acceptance PRN as a PDF</t>
-  </si>
-  <si>
-    <t>Lawrlwytho'r PRN yma sy'n aros i gael ei dderbyn fel PDF</t>
-  </si>
-  <si>
-    <t>prns.prn.downloadThisPernAwaitingAcceptance</t>
-  </si>
-  <si>
-    <t>Download this awaiting acceptance PERN as a PDF</t>
-  </si>
-  <si>
-    <t>Lawrlwytho'r PERN yma sy'n aros i gael ei dderbyn fel PDF</t>
-  </si>
-  <si>
-    <t>prns.prn.acceptanceYears</t>
-  </si>
-  <si>
-    <t>Can be accepted towards {{yearOne}} or {{yearTwo}}</t>
-  </si>
-  <si>
-    <t>prns.prn.acceptedTowardsRecyclingObligations</t>
-  </si>
-  <si>
-    <t>prns.prn.note</t>
-  </si>
-  <si>
-    <t>Note</t>
-  </si>
-  <si>
-    <t>Nodi</t>
-  </si>
-  <si>
-    <t>prns.prn.packagingExportRecyclingNote</t>
-  </si>
-  <si>
-    <t>Packaging Waste Export Recycling Note</t>
-  </si>
-  <si>
-    <t>Nodyn Ailgylchu Allforio Gwastraff Pecynwaith</t>
-  </si>
-  <si>
-    <t>prns.prn.pageTitlePern</t>
-  </si>
-  <si>
-    <t>prns.prn.pageTitlePrn</t>
-  </si>
-  <si>
-    <t>prns.prn.thisPernRelatesToWasteExportedForReprocessingInDecember</t>
-  </si>
-  <si>
-    <t>This PERN relates to waste exported for reprocessing in December {{year}}.</t>
-  </si>
-  <si>
-    <t>Mae'r PERN yma yn ymwneud â gwastraff a gafodd ei allforio i'w ailbrosesu ym mis Rhagfyr {{year}}.</t>
-  </si>
-  <si>
-    <t>prns.prn.thisPrnRelatesToWasteReceivedForReprocessingInDecember</t>
-  </si>
-  <si>
-    <t>This PRN relates to waste received for reprocessing in December {{year}}.</t>
-  </si>
-  <si>
-    <t>Mae'r PRN yma yn ymwneud â gwastraff a gafodd ei allforio i'w ailbrosesu ym mis Rhagfyr {{year}}.</t>
-  </si>
-  <si>
-    <t>prns.prn.acceptOrRejectMoreButton</t>
-  </si>
-  <si>
-    <t>Accept or reject more PRNs and PERNs for {{year}}</t>
-  </si>
-  <si>
-    <t>prns.prn.acceptOrRejectMoreButtonNoYear</t>
-  </si>
-  <si>
-    <t>Accept or reject more PRNs and PERNs</t>
-  </si>
-  <si>
-    <t>prns.prn.obligationProgressButton</t>
-  </si>
-  <si>
-    <t>View your {{year}} recycling obligations progress</t>
-  </si>
-  <si>
-    <t>prns.prn.obligationProgressButtonNoYear</t>
-  </si>
-  <si>
-    <t>View your recycling obligations progress</t>
-  </si>
-  <si>
-    <t>prns.prn.downloadThisAcceptedPrn</t>
-  </si>
-  <si>
-    <t>prns.prn.downloadThisAcceptedPern</t>
-  </si>
-  <si>
     <t>prns.prn.success.title</t>
   </si>
   <si>
@@ -430,10 +430,7 @@
     <t>prns.prn.rejected.heading</t>
   </si>
   <si>
-    <t>{{type}} rejected.</t>
-  </si>
-  <si>
-    <t>{{type}} rwrthod</t>
+    <t>You have rejected this {{type}}.</t>
   </si>
   <si>
     <t>prns.prn.agency.ea</t>
@@ -490,16 +487,16 @@
     <t>The reprocessor issued the {{prnOrPern}} to the producer or compliance scheme. The producer or compliance scheme {{meaning}}</t>
   </si>
   <si>
+    <t>prns.prn.rejected.statusMeaning</t>
+  </si>
+  <si>
+    <t>The producer or compliance scheme rejected the {{type}}.</t>
+  </si>
+  <si>
     <t>prns.prn.statusMeaningText.awaitingAcceptance</t>
   </si>
   <si>
     <t>has not yet accepted the {{prnOrPern}}.</t>
-  </si>
-  <si>
-    <t>prns.prn.statusMeaningText.rejected</t>
-  </si>
-  <si>
-    <t>has rejected the {{prnOrPern}}.</t>
   </si>
   <si>
     <t>prns.prn.statusMeaningText.cancelled</t>
@@ -1568,7 +1565,7 @@
         <v>92</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>13</v>
@@ -1576,19 +1573,19 @@
     </row>
     <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>95</v>
-      </c>
       <c r="E35" s="1" t="s">
-        <v>96</v>
+        <v>13</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>13</v>
@@ -1596,19 +1593,19 @@
     </row>
     <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>13</v>
@@ -1616,19 +1613,19 @@
     </row>
     <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E37" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>102</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>13</v>
@@ -1636,7 +1633,7 @@
     </row>
     <row r="38" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>10</v>
@@ -1645,7 +1642,7 @@
         <v>11</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>13</v>
@@ -1656,7 +1653,7 @@
     </row>
     <row r="39" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>10</v>
@@ -1676,19 +1673,19 @@
     </row>
     <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>13</v>
@@ -1696,19 +1693,19 @@
     </row>
     <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>13</v>
@@ -1716,7 +1713,7 @@
     </row>
     <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>10</v>
@@ -1736,7 +1733,7 @@
     </row>
     <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>10</v>
@@ -1756,19 +1753,19 @@
     </row>
     <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>13</v>
@@ -1776,19 +1773,19 @@
     </row>
     <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>13</v>
@@ -1796,7 +1793,7 @@
     </row>
     <row r="46" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>10</v>
@@ -1805,7 +1802,7 @@
         <v>11</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>13</v>
@@ -1816,7 +1813,7 @@
     </row>
     <row r="47" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>10</v>
@@ -1825,7 +1822,7 @@
         <v>11</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>13</v>
@@ -1836,7 +1833,7 @@
     </row>
     <row r="48" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>10</v>
@@ -1845,7 +1842,7 @@
         <v>11</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>13</v>
@@ -1856,7 +1853,7 @@
     </row>
     <row r="49" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>10</v>
@@ -1865,7 +1862,7 @@
         <v>11</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>13</v>
@@ -1876,7 +1873,7 @@
     </row>
     <row r="50" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>10</v>
@@ -1885,7 +1882,7 @@
         <v>11</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>92</v>
+        <v>127</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>13</v>
@@ -1896,16 +1893,16 @@
     </row>
     <row r="51" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>13</v>
@@ -2008,7 +2005,7 @@
         <v>139</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>140</v>
+        <v>13</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>13</v>
@@ -2016,16 +2013,16 @@
     </row>
     <row r="57" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>142</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>13</v>
@@ -2036,16 +2033,16 @@
     </row>
     <row r="58" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>13</v>
@@ -2056,16 +2053,16 @@
     </row>
     <row r="59" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>13</v>
@@ -2076,16 +2073,16 @@
     </row>
     <row r="60" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D60" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>13</v>
@@ -2096,16 +2093,16 @@
     </row>
     <row r="61" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D61" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>13</v>
@@ -2116,16 +2113,16 @@
     </row>
     <row r="62" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>13</v>
@@ -2136,16 +2133,16 @@
     </row>
     <row r="63" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>13</v>
@@ -2156,16 +2153,16 @@
     </row>
     <row r="64" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>156</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>13</v>
@@ -2176,16 +2173,16 @@
     </row>
     <row r="65" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>158</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>13</v>
@@ -2196,16 +2193,16 @@
     </row>
     <row r="66" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>13</v>
@@ -2216,16 +2213,16 @@
     </row>
     <row r="67" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>162</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>13</v>
@@ -2236,16 +2233,16 @@
     </row>
     <row r="68" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D68" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>13</v>
@@ -2256,16 +2253,16 @@
     </row>
     <row r="69" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D69" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>13</v>
@@ -2276,19 +2273,19 @@
     </row>
     <row r="70" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D70" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70" s="1" t="s">
+      <c r="E70" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="E70" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>13</v>
@@ -2296,19 +2293,19 @@
     </row>
     <row r="71" ht="64" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B71" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D71" s="1" t="s">
+      <c r="E71" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>13</v>
@@ -2316,19 +2313,19 @@
     </row>
     <row r="72" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="B72" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D72" s="1" t="s">
+      <c r="E72" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>175</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>13</v>
@@ -2336,16 +2333,16 @@
     </row>
     <row r="73" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>176</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>177</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Update PRN and PERN download button text to remove HTML option
- Changed the button text for downloading PRNs and PERNs to specify PDF format only, enhancing clarity for users.
- Updated corresponding translations in English and Welsh to reflect the change in download options.
- Adjusted related test cases to ensure consistency with the updated button text.
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
+++ b/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
@@ -289,13 +289,19 @@
     <t>prns.prn.downloadThisPrn</t>
   </si>
   <si>
-    <t>Download this PRN as a PDF or HTML</t>
+    <t>Download this PRN as a PDF</t>
+  </si>
+  <si>
+    <t>Lawrlwytho'r PRN yma fel PDF</t>
   </si>
   <si>
     <t>prns.prn.downloadThisPern</t>
   </si>
   <si>
-    <t>Download this PERN as a PDF or HTML</t>
+    <t>Download this PERN as a PDF</t>
+  </si>
+  <si>
+    <t>Lawrlwytho'r PERN yma fel PDF</t>
   </si>
   <si>
     <t>prns.prn.downloadThisPrnAwaitingAcceptance</t>
@@ -394,13 +400,7 @@
     <t>prns.prn.downloadThisAcceptedPrn</t>
   </si>
   <si>
-    <t>Download this PRN as a PDF</t>
-  </si>
-  <si>
     <t>prns.prn.downloadThisAcceptedPern</t>
-  </si>
-  <si>
-    <t>Download this PERN as a PDF</t>
   </si>
   <si>
     <t>prns.prn.success.title</t>
@@ -1565,7 +1565,7 @@
         <v>92</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>13</v>
@@ -1573,7 +1573,7 @@
     </row>
     <row r="35" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>10</v>
@@ -1582,10 +1582,10 @@
         <v>11</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>13</v>
+        <v>96</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>13</v>
@@ -1593,7 +1593,7 @@
     </row>
     <row r="36" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>10</v>
@@ -1602,10 +1602,10 @@
         <v>11</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>13</v>
@@ -1613,7 +1613,7 @@
     </row>
     <row r="37" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>10</v>
@@ -1622,10 +1622,10 @@
         <v>11</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>13</v>
@@ -1633,7 +1633,7 @@
     </row>
     <row r="38" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>10</v>
@@ -1642,7 +1642,7 @@
         <v>11</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>13</v>
@@ -1653,7 +1653,7 @@
     </row>
     <row r="39" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>10</v>
@@ -1673,7 +1673,7 @@
     </row>
     <row r="40" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>10</v>
@@ -1682,10 +1682,10 @@
         <v>11</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>13</v>
@@ -1693,7 +1693,7 @@
     </row>
     <row r="41" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>10</v>
@@ -1702,10 +1702,10 @@
         <v>11</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>13</v>
@@ -1713,7 +1713,7 @@
     </row>
     <row r="42" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>10</v>
@@ -1733,7 +1733,7 @@
     </row>
     <row r="43" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>10</v>
@@ -1753,7 +1753,7 @@
     </row>
     <row r="44" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>10</v>
@@ -1762,10 +1762,10 @@
         <v>11</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>13</v>
@@ -1773,7 +1773,7 @@
     </row>
     <row r="45" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>10</v>
@@ -1782,10 +1782,10 @@
         <v>11</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>13</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="46" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>10</v>
@@ -1802,7 +1802,7 @@
         <v>11</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>13</v>
@@ -1813,7 +1813,7 @@
     </row>
     <row r="47" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>10</v>
@@ -1822,7 +1822,7 @@
         <v>11</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>13</v>
@@ -1833,7 +1833,7 @@
     </row>
     <row r="48" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>10</v>
@@ -1842,7 +1842,7 @@
         <v>11</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>13</v>
@@ -1853,7 +1853,7 @@
     </row>
     <row r="49" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>10</v>
@@ -1862,7 +1862,7 @@
         <v>11</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>13</v>
@@ -1873,7 +1873,7 @@
     </row>
     <row r="50" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>10</v>
@@ -1882,7 +1882,7 @@
         <v>11</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>127</v>
+        <v>92</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>13</v>
@@ -1893,7 +1893,7 @@
     </row>
     <row r="51" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>10</v>
@@ -1902,7 +1902,7 @@
         <v>11</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>129</v>
+        <v>95</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Update December waste terminology in English and Welsh translations
- Changed "December waste?" to "December Waste?" for consistency in capitalization.
- Updated responses for "isDecemberWaste" and "isNotDecemberWaste" to lowercase "yes" and "no" respectively.
- Adjusted related test cases to reflect these changes in the UI and translations.
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
+++ b/translations/welsh-translations/xlsx/14-producer-prns-prn.xlsx
@@ -181,7 +181,7 @@
     <t>prns.prn.relatesToWasteReceivedInDecember</t>
   </si>
   <si>
-    <t>December waste?</t>
+    <t>December Waste?</t>
   </si>
   <si>
     <t>Gwastraff Rhagfyr?</t>
@@ -190,7 +190,7 @@
     <t>prns.prn.isDecemberWaste</t>
   </si>
   <si>
-    <t>Yes</t>
+    <t>yes</t>
   </si>
   <si>
     <t>Ydw</t>
@@ -199,7 +199,7 @@
     <t>prns.prn.isNotDecemberWaste</t>
   </si>
   <si>
-    <t>No</t>
+    <t>no</t>
   </si>
   <si>
     <t>Nac ydw</t>

</xml_diff>